<commit_message>
TED-MDB 1927 with CoNLL-U segmentation
</commit_message>
<xml_diff>
--- a/scripts/ted-mdb-1927.xlsx
+++ b/scripts/ted-mdb-1927.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1234" uniqueCount="311">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1283" uniqueCount="318">
   <si>
     <t>ID</t>
   </si>
@@ -52,16 +52,34 @@
     <t>_</t>
   </si>
   <si>
-    <t>talkid: 1927 Chris McKnett: The investment logic for sustainability The world is changing in some really profound ways, and I worry that investors aren't paying enough attention to some of the biggest drivers of change, especially when it comes to sustainability.</t>
+    <t>talkid: 1927</t>
   </si>
   <si>
     <t>2</t>
   </si>
   <si>
+    <t>Chris McKnett:</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>The investment logic for sustainability</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>The world is changing in some really profound ways, and I worry that investors aren't paying enough attention to some of the biggest drivers of change, especially when it comes to sustainability.</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
     <t>And by sustainability, I mean the really juicy things, like environmental and social issues and corporate governance.</t>
   </si>
   <si>
-    <t>3</t>
+    <t>6</t>
   </si>
   <si>
     <t>(in fact)</t>
@@ -79,7 +97,7 @@
     <t>(orig: Expansion.Level-of-detail.Arg2-as-detail)</t>
   </si>
   <si>
-    <t>4</t>
+    <t>7</t>
   </si>
   <si>
     <t>And here's something that may surprise you: the balance of power to really influence sustainability rests with institutional investors, the large investors like pension funds, foundations and endowments.</t>
@@ -94,19 +112,19 @@
     <t>(orig: Expansion.Conjunction)</t>
   </si>
   <si>
-    <t>5</t>
+    <t>8</t>
   </si>
   <si>
     <t>I believe that sustainable investing is less complicated than you think, better-performing than you believe, and more important than we can imagine.</t>
   </si>
   <si>
-    <t>6</t>
+    <t>9</t>
   </si>
   <si>
     <t>Let me remind you what we already know.</t>
   </si>
   <si>
-    <t>7</t>
+    <t>10</t>
   </si>
   <si>
     <t>(that is)</t>
@@ -115,13 +133,13 @@
     <t>We have a population that's both growing and aging; we have seven billion souls today heading to 10 billion at the end of the century; we consume natural resources faster than they can be replenished; and the emissions that are mainly responsible for climate change just keep increasing.</t>
   </si>
   <si>
-    <t>8</t>
+    <t>11</t>
   </si>
   <si>
     <t>Now clearly, these are environmental and social issues, but that's not all.</t>
   </si>
   <si>
-    <t>9</t>
+    <t>12</t>
   </si>
   <si>
     <t>(additionally)</t>
@@ -130,13 +148,13 @@
     <t>They're economic issues, and that makes them relevant to risk and return.</t>
   </si>
   <si>
-    <t>10</t>
+    <t>13</t>
   </si>
   <si>
     <t>And they are really complex and they can seem really far off, that the temptation may be to do this: bury our heads in the sand and not think about it.</t>
   </si>
   <si>
-    <t>11</t>
+    <t>14</t>
   </si>
   <si>
     <t>(but)</t>
@@ -154,7 +172,7 @@
     <t>(orig: Comparison.Contrast)</t>
   </si>
   <si>
-    <t>12</t>
+    <t>15</t>
   </si>
   <si>
     <t>(in other words)</t>
@@ -163,13 +181,19 @@
     <t>Don't do this at home.</t>
   </si>
   <si>
-    <t>13</t>
-  </si>
-  <si>
-    <t>(Laughter) But it makes me wonder if the investment rules of today are fit for purpose tomorrow.</t>
-  </si>
-  <si>
-    <t>14</t>
+    <t>16</t>
+  </si>
+  <si>
+    <t>(Laughter)</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>But it makes me wonder if the investment rules of today are fit for purpose tomorrow.</t>
+  </si>
+  <si>
+    <t>18</t>
   </si>
   <si>
     <t>(for example)</t>
@@ -187,13 +211,13 @@
     <t>(orig: Expansion.Instantiation)</t>
   </si>
   <si>
-    <t>15</t>
+    <t>19</t>
   </si>
   <si>
     <t>And these things are fundamental, of course, but they're not enough.</t>
   </si>
   <si>
-    <t>16</t>
+    <t>20</t>
   </si>
   <si>
     <t>(because)</t>
@@ -205,19 +229,19 @@
     <t>Contingency.Cause+Belief.Reason+Belief</t>
   </si>
   <si>
-    <t>causal+reason</t>
+    <t>causal|reason</t>
   </si>
   <si>
     <t>(orig: Contingency.Cause+Belief.Reason+Belief)</t>
   </si>
   <si>
-    <t>17</t>
+    <t>21</t>
   </si>
   <si>
     <t>Environment includes energy consumption, water availability, waste and pollution, just making efficient uses of resources.</t>
   </si>
   <si>
-    <t>18</t>
+    <t>22</t>
   </si>
   <si>
     <t>(and)</t>
@@ -226,13 +250,13 @@
     <t>Social includes human capital, things like employee engagement and innovation capacity, as well as supply chain management and labor rights and human rights.</t>
   </si>
   <si>
-    <t>19</t>
+    <t>23</t>
   </si>
   <si>
     <t>And governance relates to the oversight of companies by their boards and investors.</t>
   </si>
   <si>
-    <t>20</t>
+    <t>24</t>
   </si>
   <si>
     <t>See, I told you this is the really juicy stuff.</t>
@@ -241,13 +265,13 @@
     <t>Contingency.Cause+SpeechAct.Result+SpeechAct</t>
   </si>
   <si>
-    <t>causal+result</t>
+    <t>causal|result</t>
   </si>
   <si>
     <t>(orig: Contingency.Cause+SpeechAct.Result+SpeechAct)</t>
   </si>
   <si>
-    <t>21</t>
+    <t>25</t>
   </si>
   <si>
     <t>But ESG is the measure of sustainability, and sustainable investing incorporates ESG factors with financial factors into the investment process.</t>
@@ -262,7 +286,7 @@
     <t>(orig: Comparison.Concession.Arg2-as-denier)</t>
   </si>
   <si>
-    <t>22</t>
+    <t>26</t>
   </si>
   <si>
     <t>It means limiting future risk by minimizing harm to people and planet, and it means providing capital to users who deploy it towards productive and sustainable outcomes.</t>
@@ -277,19 +301,19 @@
     <t>(orig: Expansion.Equivalence)</t>
   </si>
   <si>
-    <t>23</t>
+    <t>27</t>
   </si>
   <si>
     <t>So if sustainability matters financially today, and all signs indicate more tomorrow, is the private sector paying attention?</t>
   </si>
   <si>
-    <t>24</t>
+    <t>28</t>
   </si>
   <si>
     <t>Well, the really cool thing is that most CEOs are.</t>
   </si>
   <si>
-    <t>25</t>
+    <t>29</t>
   </si>
   <si>
     <t>(specifically)</t>
@@ -298,25 +322,25 @@
     <t>They started to see sustainability not just as important but crucial to business success.</t>
   </si>
   <si>
-    <t>26</t>
+    <t>30</t>
   </si>
   <si>
     <t>About 80 percent of global CEOs see sustainability as the root to growth in innovation and leading to competitive advantage in their industries.</t>
   </si>
   <si>
-    <t>27</t>
+    <t>31</t>
   </si>
   <si>
     <t>But 93 percent see ESG as the future, or as important to the future of their business.</t>
   </si>
   <si>
-    <t>28</t>
+    <t>32</t>
   </si>
   <si>
     <t>So the views of CEOs are clear.</t>
   </si>
   <si>
-    <t>29</t>
+    <t>33</t>
   </si>
   <si>
     <t>(in sum)</t>
@@ -325,31 +349,31 @@
     <t>There's tremendous opportunity in sustainability.</t>
   </si>
   <si>
-    <t>30</t>
+    <t>34</t>
   </si>
   <si>
     <t>So how are companies actually leveraging ESG to drive hard business results?</t>
   </si>
   <si>
-    <t>31</t>
+    <t>35</t>
   </si>
   <si>
     <t>One example is near and dear to our hearts.</t>
   </si>
   <si>
-    <t>32</t>
+    <t>36</t>
   </si>
   <si>
     <t>In 2012, State Street migrated 54 applications to the cloud environment, and we retired another 85.</t>
   </si>
   <si>
-    <t>33</t>
+    <t>37</t>
   </si>
   <si>
     <t>We virtualized our operating system environments, and we completed numerous automation projects.</t>
   </si>
   <si>
-    <t>34</t>
+    <t>38</t>
   </si>
   <si>
     <t>Now these initiatives create a more mobile workplace, and they reduce our real estate footprint, and they yield savings of 23 million dollars in operating costs annually, and avoid the emissions of a 100,000 metric tons of carbon.</t>
@@ -364,49 +388,43 @@
     <t>(orig: Contingency.Cause.Result)</t>
   </si>
   <si>
-    <t>35</t>
+    <t>39</t>
   </si>
   <si>
     <t>That's the equivalent of taking 21,000 cars off the road.</t>
   </si>
   <si>
-    <t>36</t>
+    <t>40</t>
   </si>
   <si>
     <t>So awesome, right?</t>
   </si>
   <si>
-    <t>37</t>
+    <t>41</t>
   </si>
   <si>
     <t>Another example is Pentair.</t>
   </si>
   <si>
-    <t>38</t>
-  </si>
-  <si>
-    <t>Pentair is a U.S.</t>
-  </si>
-  <si>
-    <t>39</t>
-  </si>
-  <si>
-    <t>industrial conglomerate, and about a decade ago, they sold their core power tools business and reinvested those proceeds in a water business.</t>
-  </si>
-  <si>
-    <t>40</t>
+    <t>42</t>
+  </si>
+  <si>
+    <t>Pentair is a U.S. industrial conglomerate, and about a decade ago, they sold their core power tools business and reinvested those proceeds in a water business.</t>
+  </si>
+  <si>
+    <t>43</t>
   </si>
   <si>
     <t>That's a really big bet.</t>
   </si>
   <si>
-    <t>41</t>
+    <t>44</t>
   </si>
   <si>
     <t>Why did they do that?</t>
   </si>
   <si>
-    <t>42</t>
+    <t>45</t>
   </si>
   <si>
     <t>Hypophora</t>
@@ -424,61 +442,61 @@
     <t>(orig: Contingency.Cause.Reason)</t>
   </si>
   <si>
-    <t>43</t>
+    <t>46</t>
   </si>
   <si>
     <t>That's four billion middle class people demanding food, energy and water.</t>
   </si>
   <si>
-    <t>44</t>
+    <t>47</t>
   </si>
   <si>
     <t>Now, you may be asking yourself, are these just isolated cases?</t>
   </si>
   <si>
-    <t>45</t>
+    <t>48</t>
   </si>
   <si>
     <t>I mean, come on, really?</t>
   </si>
   <si>
-    <t>46</t>
+    <t>49</t>
   </si>
   <si>
     <t>Do companies that take sustainability into account really do well financially?</t>
   </si>
   <si>
-    <t>47</t>
+    <t>50</t>
   </si>
   <si>
     <t>The answer that may surprise you is yes.</t>
   </si>
   <si>
-    <t>48</t>
+    <t>51</t>
   </si>
   <si>
     <t>The data shows that stocks with better ESG performance perform just as well as others.</t>
   </si>
   <si>
-    <t>49</t>
+    <t>52</t>
   </si>
   <si>
     <t>In blue, we see the MSCI World.</t>
   </si>
   <si>
-    <t>50</t>
+    <t>53</t>
   </si>
   <si>
     <t>It's an index of large companies from developed markets across the world.</t>
   </si>
   <si>
-    <t>51</t>
+    <t>54</t>
   </si>
   <si>
     <t>And in gold, we see a subset of companies rated as having the best ESG performance.</t>
   </si>
   <si>
-    <t>52</t>
+    <t>55</t>
   </si>
   <si>
     <t>(in short)</t>
@@ -496,19 +514,19 @@
     <t>(orig: Expansion.Level-of-detail.Arg1-as-detail)</t>
   </si>
   <si>
-    <t>53</t>
+    <t>56</t>
   </si>
   <si>
     <t>So that's okay, right?</t>
   </si>
   <si>
-    <t>54</t>
+    <t>57</t>
   </si>
   <si>
     <t>We want more.</t>
   </si>
   <si>
-    <t>55</t>
+    <t>58</t>
   </si>
   <si>
     <t>(furthermore)</t>
@@ -517,13 +535,13 @@
     <t>I want more.</t>
   </si>
   <si>
-    <t>56</t>
+    <t>59</t>
   </si>
   <si>
     <t>In some cases, there may be outperformance from ESG.</t>
   </si>
   <si>
-    <t>57</t>
+    <t>60</t>
   </si>
   <si>
     <t>(for instance)</t>
@@ -532,7 +550,7 @@
     <t>In blue, we see the performance of the 500 largest global companies, and in gold, we see a subset of companies with best practice in climate change strategy and risk management.</t>
   </si>
   <si>
-    <t>58</t>
+    <t>61</t>
   </si>
   <si>
     <t>(clearly)</t>
@@ -541,13 +559,13 @@
     <t>Now over almost eight years, they've outperformed by about two thirds.</t>
   </si>
   <si>
-    <t>59</t>
+    <t>62</t>
   </si>
   <si>
     <t>So yes, this is correlation.</t>
   </si>
   <si>
-    <t>60</t>
+    <t>63</t>
   </si>
   <si>
     <t>(rather)</t>
@@ -565,49 +583,49 @@
     <t>(orig: Expansion.Substitution.Arg1-as-subst)</t>
   </si>
   <si>
-    <t>61</t>
+    <t>64</t>
   </si>
   <si>
     <t>But it does illustrate that environmental leadership is compatible with good returns.</t>
   </si>
   <si>
-    <t>62</t>
+    <t>65</t>
   </si>
   <si>
     <t>So if the returns are the same or better and the planet benefits, wouldn't this be the norm?</t>
   </si>
   <si>
-    <t>63</t>
+    <t>66</t>
   </si>
   <si>
     <t>Are investors, particularly institutional investors, engaged?</t>
   </si>
   <si>
-    <t>64</t>
+    <t>67</t>
   </si>
   <si>
     <t>Well, some are, and a few are really at the vanguard.</t>
   </si>
   <si>
-    <t>65</t>
+    <t>68</t>
   </si>
   <si>
     <t>Hesta.</t>
   </si>
   <si>
-    <t>66</t>
+    <t>69</t>
   </si>
   <si>
     <t>Hesta is a retirement fund for health and community services employees in Australia, with assets of 22 billion [dollars].</t>
   </si>
   <si>
-    <t>67</t>
+    <t>70</t>
   </si>
   <si>
     <t>They believe that ESG has the potential to impact risks and returns, so incorporating it into the investment process is core to their duty to act in the best interest of fund members, core to their duty.</t>
   </si>
   <si>
-    <t>68</t>
+    <t>71</t>
   </si>
   <si>
     <t>(so)</t>
@@ -616,49 +634,43 @@
     <t>You gotta love the Aussies, right?</t>
   </si>
   <si>
-    <t>69</t>
+    <t>72</t>
   </si>
   <si>
     <t>CalPERS is another example.</t>
   </si>
   <si>
-    <t>70</t>
-  </si>
-  <si>
-    <t>CalPERS is the pension fund for public employees in California, and with assets of 244 billion [dollars], they are the second largest in the U.S.</t>
-  </si>
-  <si>
-    <t>71</t>
-  </si>
-  <si>
-    <t>and the sixth largest in the world.</t>
-  </si>
-  <si>
-    <t>72</t>
+    <t>73</t>
+  </si>
+  <si>
+    <t>CalPERS is the pension fund for public employees in California, and with assets of 244 billion [dollars], they are the second largest in the U.S. and the sixth largest in the world.</t>
+  </si>
+  <si>
+    <t>74</t>
   </si>
   <si>
     <t>Now, they're moving toward 100 percent sustainable investment by systematically integrated ESG across the entire fund.</t>
   </si>
   <si>
-    <t>73</t>
+    <t>75</t>
   </si>
   <si>
     <t>Why?</t>
   </si>
   <si>
-    <t>74</t>
+    <t>76</t>
   </si>
   <si>
     <t>They believe it's critical to superior long-term returns, full stop.</t>
   </si>
   <si>
-    <t>75</t>
+    <t>77</t>
   </si>
   <si>
     <t>In their own words, "long-term value creation requires the effective management of three forms of capital: financial, human, and physical.</t>
   </si>
   <si>
-    <t>76</t>
+    <t>78</t>
   </si>
   <si>
     <t>This is why we are concerned with ESG."</t>
@@ -670,7 +682,7 @@
     <t>(orig: Contingency.Cause+Belief.Result+Belief)</t>
   </si>
   <si>
-    <t>77</t>
+    <t>79</t>
   </si>
   <si>
     <t>(however)</t>
@@ -679,7 +691,7 @@
     <t>Now, I do speak to a lot of investors as part of my job, and not all of them see it this way.</t>
   </si>
   <si>
-    <t>78</t>
+    <t>80</t>
   </si>
   <si>
     <t>(instead)</t>
@@ -697,103 +709,112 @@
     <t>(orig: Expansion.Substitution.Arg2-as-subst)</t>
   </si>
   <si>
-    <t>79</t>
-  </si>
-  <si>
-    <t>The one that just really gets under my skin is, "If you want to do something about that, just make money, give the profits to charities."</t>
-  </si>
-  <si>
-    <t>80</t>
+    <t>81</t>
+  </si>
+  <si>
+    <t>The one that just really gets under my skin is,</t>
+  </si>
+  <si>
+    <t>82</t>
+  </si>
+  <si>
+    <t>"If you want to do something about that, just make money, give the profits to charities."</t>
+  </si>
+  <si>
+    <t>83</t>
   </si>
   <si>
     <t>It's eyes rolling, eyes rolling.</t>
   </si>
   <si>
-    <t>81</t>
+    <t>84</t>
   </si>
   <si>
     <t>I mean, let me clarify something right here.</t>
   </si>
   <si>
-    <t>82</t>
+    <t>85</t>
   </si>
   <si>
     <t>Companies and investors are not singularly responsible for the fate of the planet.</t>
   </si>
   <si>
-    <t>83</t>
+    <t>86</t>
   </si>
   <si>
     <t>They don't have indefinite social obligations, and prudent investing and finance theory aren't subordinate to sustainability.</t>
   </si>
   <si>
-    <t>84</t>
+    <t>87</t>
   </si>
   <si>
     <t>They're compatible.</t>
   </si>
   <si>
-    <t>85</t>
+    <t>88</t>
   </si>
   <si>
     <t>So I'm not talking about tradeoffs here.</t>
   </si>
   <si>
-    <t>86</t>
+    <t>89</t>
   </si>
   <si>
     <t>But institutional investors are the x-factor in sustainability.</t>
   </si>
   <si>
-    <t>87</t>
+    <t>90</t>
   </si>
   <si>
     <t>Why do they hold the key?</t>
   </si>
   <si>
-    <t>88</t>
+    <t>91</t>
   </si>
   <si>
     <t>The answer, quite simply, is, they have the money.</t>
   </si>
   <si>
-    <t>89</t>
-  </si>
-  <si>
-    <t>(Laughter) A lot of it.</t>
-  </si>
-  <si>
-    <t>90</t>
+    <t>92</t>
+  </si>
+  <si>
+    <t>93</t>
+  </si>
+  <si>
+    <t>A lot of it.</t>
+  </si>
+  <si>
+    <t>94</t>
   </si>
   <si>
     <t>I mean, a really lot of it.</t>
   </si>
   <si>
-    <t>91</t>
+    <t>95</t>
   </si>
   <si>
     <t>The global stock market is worth 55 trillion dollars.</t>
   </si>
   <si>
-    <t>92</t>
+    <t>96</t>
   </si>
   <si>
     <t>The global bond market, 78 trillion.</t>
   </si>
   <si>
-    <t>93</t>
+    <t>97</t>
   </si>
   <si>
     <t>That's 133 trillion combined.</t>
   </si>
   <si>
-    <t>94</t>
+    <t>98</t>
   </si>
   <si>
     <t>(by comparison)</t>
   </si>
   <si>
-    <t>That's eight and a half times the GDP of the U.S.</t>
+    <t>That's eight and a half times the GDP of the U.S. That's the world's largest economy.</t>
   </si>
   <si>
     <t>Comparison.Similarity</t>
@@ -805,67 +826,55 @@
     <t>(orig: Comparison.Similarity)</t>
   </si>
   <si>
-    <t>95</t>
-  </si>
-  <si>
-    <t>That's the world's largest economy.</t>
-  </si>
-  <si>
-    <t>96</t>
+    <t>99</t>
   </si>
   <si>
     <t>That's some serious freaking firepower.</t>
   </si>
   <si>
-    <t>97</t>
+    <t>100</t>
   </si>
   <si>
     <t>So we can reconsider some of these pressing challenges, like fresh water, clean air, feeding 10 billion mouths, if institutional investors integrated ESG into investment.</t>
   </si>
   <si>
-    <t>98</t>
+    <t>101</t>
   </si>
   <si>
     <t>What if they used that firepower to allocate more of their capital to companies working the hardest at solving these challenges or at least not exacerbating them?</t>
   </si>
   <si>
-    <t>99</t>
+    <t>102</t>
   </si>
   <si>
     <t>What if we work and save and invest, only to find that the world we retire into is more stressed and less secure than it is now?</t>
   </si>
   <si>
-    <t>100</t>
+    <t>103</t>
   </si>
   <si>
     <t>What if there isn't enough clean air and fresh water?</t>
   </si>
   <si>
-    <t>101</t>
+    <t>104</t>
   </si>
   <si>
     <t>Now a fair question might be, what if all this sustainability risk stuff is exaggerated, overstated, it's not urgent, something for virtuous consumers or lifestyle choice?</t>
   </si>
   <si>
-    <t>103</t>
-  </si>
-  <si>
-    <t>102</t>
-  </si>
-  <si>
-    <t>Well, President John F.</t>
-  </si>
-  <si>
-    <t>Kennedy said something about this that is just spot on: "There are risks and costs to a program of action, but they are far less than the long-range risks and costs of comfortable inaction."</t>
-  </si>
-  <si>
-    <t>104</t>
+    <t>105</t>
+  </si>
+  <si>
+    <t>Well, President John F. Kennedy said something about this that is just spot on: "There are risks and costs to a program of action, but they are far less than the long-range risks and costs of comfortable inaction."</t>
+  </si>
+  <si>
+    <t>106</t>
   </si>
   <si>
     <t>I can appreciate that there is estimation risk in this, but since this is based on widespread scientific consensus, the odds that it's not completely wrong are better than the odds that our house will burn down or we'll get in a car accident.</t>
   </si>
   <si>
-    <t>105</t>
+    <t>107</t>
   </si>
   <si>
     <t>(except)</t>
@@ -883,19 +892,22 @@
     <t>(orig: Expansion.Exception.Arg2-as-excpt)</t>
   </si>
   <si>
-    <t>106</t>
-  </si>
-  <si>
-    <t>(Laughter) But my point is that we buy insurance to protect ourselves financially in case those things happen, right?</t>
-  </si>
-  <si>
-    <t>107</t>
+    <t>108</t>
+  </si>
+  <si>
+    <t>109</t>
+  </si>
+  <si>
+    <t>But my point is that we buy insurance to protect ourselves financially in case those things happen, right?</t>
+  </si>
+  <si>
+    <t>110</t>
   </si>
   <si>
     <t>So by investing sustainably we're doing two things.</t>
   </si>
   <si>
-    <t>108</t>
+    <t>111</t>
   </si>
   <si>
     <t>(namely)</t>
@@ -904,19 +916,25 @@
     <t>We're creating insurance, reducing the risk to our planet and to our economy, and at the same time, in the short term, we're not sacrificing performance.</t>
   </si>
   <si>
-    <t>109</t>
-  </si>
-  <si>
-    <t>[Man in comic: "What if it's a big hoax and we create a better world for nothing?"]</t>
-  </si>
-  <si>
-    <t>110</t>
+    <t>112</t>
+  </si>
+  <si>
+    <t>[Man in comic:</t>
+  </si>
+  <si>
+    <t>113</t>
+  </si>
+  <si>
+    <t>"What if it's a big hoax and we create a better world for nothing?"]</t>
+  </si>
+  <si>
+    <t>114</t>
   </si>
   <si>
     <t>Good, you like it.</t>
   </si>
   <si>
-    <t>111</t>
+    <t>115</t>
   </si>
   <si>
     <t>(for that matter)</t>
@@ -925,25 +943,28 @@
     <t>I like it too.</t>
   </si>
   <si>
-    <t>112</t>
-  </si>
-  <si>
-    <t>(Laughter) I like it because it pokes fun at both sides of the climate change issue.</t>
-  </si>
-  <si>
-    <t>113</t>
+    <t>116</t>
+  </si>
+  <si>
+    <t>117</t>
+  </si>
+  <si>
+    <t>I like it because it pokes fun at both sides of the climate change issue.</t>
+  </si>
+  <si>
+    <t>118</t>
   </si>
   <si>
     <t>I bet you can't guess which side I'm on.</t>
   </si>
   <si>
-    <t>114</t>
+    <t>119</t>
   </si>
   <si>
     <t>But what I really like about it is that it reminds me of something Mark Twain said, which is, "Plan for the future, because that's where you're going to spend the rest of your life."</t>
   </si>
   <si>
-    <t>115</t>
+    <t>120</t>
   </si>
   <si>
     <t>Thank you.</t>
@@ -1351,7 +1372,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J116"/>
+  <dimension ref="A1:J121"/>
   <sheetFormatPr defaultRowHeight="60" customHeight="1"/>
   <cols>
     <col min="2" max="3" width="0" hidden="1" customWidth="1"/>
@@ -1465,13 +1486,13 @@
         <v>11</v>
       </c>
       <c r="C4" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" s="8" t="s">
         <v>16</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>17</v>
       </c>
       <c r="F4" s="6" t="s">
         <v>11</v>
@@ -1481,18 +1502,16 @@
         <v/>
       </c>
       <c r="H4" s="10" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="I4" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="J4" s="12" t="s">
-        <v>20</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="J4" s="12"/>
     </row>
     <row r="5" spans="1:10" ht="60" customHeight="1">
       <c r="A5" s="6" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>11</v>
@@ -1504,7 +1523,7 @@
         <v>11</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>11</v>
@@ -1514,30 +1533,28 @@
         <v/>
       </c>
       <c r="H5" s="10" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="J5" s="12" t="s">
-        <v>25</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="J5" s="12"/>
     </row>
     <row r="6" spans="1:10" ht="60" customHeight="1">
       <c r="A6" s="6" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F6" s="6" t="s">
         <v>11</v>
@@ -1547,30 +1564,28 @@
         <v/>
       </c>
       <c r="H6" s="10" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="J6" s="12" t="s">
-        <v>20</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="J6" s="12"/>
     </row>
     <row r="7" spans="1:10" ht="60" customHeight="1">
       <c r="A7" s="6" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="F7" s="6" t="s">
         <v>11</v>
@@ -1580,28 +1595,30 @@
         <v/>
       </c>
       <c r="H7" s="10" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="I7" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="J7" s="12"/>
+        <v>25</v>
+      </c>
+      <c r="J7" s="12" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="8" spans="1:10" ht="60" customHeight="1">
       <c r="A8" s="6" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>11</v>
@@ -1611,30 +1628,30 @@
         <v/>
       </c>
       <c r="H8" s="10" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="I8" s="11" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="J8" s="12" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="60" customHeight="1">
       <c r="A9" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="8" t="s">
         <v>33</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>34</v>
       </c>
       <c r="F9" s="6" t="s">
         <v>11</v>
@@ -1644,30 +1661,30 @@
         <v/>
       </c>
       <c r="H9" s="10" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="I9" s="11" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="J9" s="12" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="60" customHeight="1">
       <c r="A10" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" s="8" t="s">
         <v>35</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>37</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>11</v>
@@ -1677,30 +1694,28 @@
         <v/>
       </c>
       <c r="H10" s="10" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="I10" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="J10" s="12" t="s">
-        <v>20</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="J10" s="12"/>
     </row>
     <row r="11" spans="1:10" ht="60" customHeight="1">
       <c r="A11" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" s="8" t="s">
         <v>38</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" s="8" t="s">
-        <v>39</v>
       </c>
       <c r="F11" s="6" t="s">
         <v>11</v>
@@ -1710,30 +1725,30 @@
         <v/>
       </c>
       <c r="H11" s="10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I11" s="11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J11" s="12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="60" customHeight="1">
       <c r="A12" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" s="8" t="s">
         <v>40</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E12" s="8" t="s">
-        <v>42</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>11</v>
@@ -1743,30 +1758,30 @@
         <v/>
       </c>
       <c r="H12" s="10" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="I12" s="11" t="s">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="J12" s="12" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="60" customHeight="1">
       <c r="A13" s="6" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="D13" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="F13" s="6" t="s">
         <v>11</v>
@@ -1776,18 +1791,18 @@
         <v/>
       </c>
       <c r="H13" s="10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I13" s="11" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="J13" s="12" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="60" customHeight="1">
       <c r="A14" s="6" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>11</v>
@@ -1799,7 +1814,7 @@
         <v>11</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>11</v>
@@ -1809,30 +1824,30 @@
         <v/>
       </c>
       <c r="H14" s="10" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="I14" s="11" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="J14" s="12" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="60" customHeight="1">
       <c r="A15" s="6" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="F15" s="6" t="s">
         <v>11</v>
@@ -1842,30 +1857,30 @@
         <v/>
       </c>
       <c r="H15" s="10" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="I15" s="11" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="J15" s="12" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="60" customHeight="1">
       <c r="A16" s="6" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>11</v>
+        <v>53</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>11</v>
@@ -1875,30 +1890,30 @@
         <v/>
       </c>
       <c r="H16" s="10" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="I16" s="11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J16" s="12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="60" customHeight="1">
       <c r="A17" s="6" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>60</v>
+        <v>11</v>
       </c>
       <c r="D17" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="F17" s="6" t="s">
         <v>11</v>
@@ -1908,18 +1923,16 @@
         <v/>
       </c>
       <c r="H17" s="10" t="s">
-        <v>57</v>
+        <v>11</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="J17" s="12" t="s">
-        <v>64</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="J17" s="12"/>
     </row>
     <row r="18" spans="1:10" ht="60" customHeight="1">
       <c r="A18" s="6" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>11</v>
@@ -1931,7 +1944,7 @@
         <v>11</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>11</v>
@@ -1941,28 +1954,30 @@
         <v/>
       </c>
       <c r="H18" s="10" t="s">
-        <v>11</v>
+        <v>44</v>
       </c>
       <c r="I18" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="J18" s="12"/>
+        <v>25</v>
+      </c>
+      <c r="J18" s="12" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="19" spans="1:10" ht="60" customHeight="1">
       <c r="A19" s="6" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="B19" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="D19" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="F19" s="6" t="s">
         <v>11</v>
@@ -1972,18 +1987,18 @@
         <v/>
       </c>
       <c r="H19" s="10" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="I19" s="11" t="s">
-        <v>24</v>
+        <v>63</v>
       </c>
       <c r="J19" s="12" t="s">
-        <v>25</v>
+        <v>64</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="60" customHeight="1">
       <c r="A20" s="6" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>11</v>
@@ -1995,7 +2010,7 @@
         <v>11</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>11</v>
@@ -2005,30 +2020,30 @@
         <v/>
       </c>
       <c r="H20" s="10" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="I20" s="11" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="J20" s="12" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="60" customHeight="1">
       <c r="A21" s="6" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="B21" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>11</v>
+        <v>68</v>
       </c>
       <c r="D21" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="F21" s="6" t="s">
         <v>11</v>
@@ -2038,18 +2053,18 @@
         <v/>
       </c>
       <c r="H21" s="10" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="I21" s="11" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="J21" s="12" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="60" customHeight="1">
       <c r="A22" s="6" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B22" s="6" t="s">
         <v>11</v>
@@ -2061,7 +2076,7 @@
         <v>11</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>11</v>
@@ -2071,30 +2086,28 @@
         <v/>
       </c>
       <c r="H22" s="10" t="s">
-        <v>72</v>
+        <v>11</v>
       </c>
       <c r="I22" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="J22" s="12" t="s">
-        <v>81</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="J22" s="12"/>
     </row>
     <row r="23" spans="1:10" ht="60" customHeight="1">
       <c r="A23" s="6" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>11</v>
+        <v>76</v>
       </c>
       <c r="D23" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="F23" s="6" t="s">
         <v>11</v>
@@ -2104,18 +2117,18 @@
         <v/>
       </c>
       <c r="H23" s="10" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="I23" s="11" t="s">
-        <v>85</v>
+        <v>30</v>
       </c>
       <c r="J23" s="12" t="s">
-        <v>86</v>
+        <v>31</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="60" customHeight="1">
       <c r="A24" s="6" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B24" s="6" t="s">
         <v>11</v>
@@ -2127,7 +2140,7 @@
         <v>11</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>11</v>
@@ -2137,18 +2150,18 @@
         <v/>
       </c>
       <c r="H24" s="10" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="I24" s="11" t="s">
-        <v>75</v>
+        <v>30</v>
       </c>
       <c r="J24" s="12" t="s">
-        <v>76</v>
+        <v>31</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="60" customHeight="1">
       <c r="A25" s="6" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>11</v>
@@ -2160,7 +2173,7 @@
         <v>11</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="F25" s="6" t="s">
         <v>11</v>
@@ -2170,28 +2183,30 @@
         <v/>
       </c>
       <c r="H25" s="10" t="s">
-        <v>11</v>
+        <v>75</v>
       </c>
       <c r="I25" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="J25" s="12"/>
+        <v>83</v>
+      </c>
+      <c r="J25" s="12" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="26" spans="1:10" ht="60" customHeight="1">
       <c r="A26" s="6" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="B26" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>92</v>
+        <v>11</v>
       </c>
       <c r="D26" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>11</v>
@@ -2201,30 +2216,30 @@
         <v/>
       </c>
       <c r="H26" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="I26" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="J26" s="12" t="s">
         <v>89</v>
-      </c>
-      <c r="I26" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="J26" s="12" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="60" customHeight="1">
       <c r="A27" s="6" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B27" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D27" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="F27" s="6" t="s">
         <v>11</v>
@@ -2234,30 +2249,30 @@
         <v/>
       </c>
       <c r="H27" s="10" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="I27" s="11" t="s">
-        <v>19</v>
+        <v>93</v>
       </c>
       <c r="J27" s="12" t="s">
-        <v>20</v>
+        <v>94</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="60" customHeight="1">
       <c r="A28" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E28" s="8" t="s">
         <v>96</v>
-      </c>
-      <c r="B28" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C28" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D28" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E28" s="8" t="s">
-        <v>97</v>
       </c>
       <c r="F28" s="6" t="s">
         <v>11</v>
@@ -2267,30 +2282,30 @@
         <v/>
       </c>
       <c r="H28" s="10" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="I28" s="11" t="s">
-        <v>44</v>
+        <v>83</v>
       </c>
       <c r="J28" s="12" t="s">
-        <v>45</v>
+        <v>84</v>
       </c>
     </row>
     <row r="29" spans="1:10" ht="60" customHeight="1">
       <c r="A29" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E29" s="8" t="s">
         <v>98</v>
-      </c>
-      <c r="B29" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C29" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D29" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E29" s="8" t="s">
-        <v>99</v>
       </c>
       <c r="F29" s="6" t="s">
         <v>11</v>
@@ -2300,30 +2315,28 @@
         <v/>
       </c>
       <c r="H29" s="10" t="s">
-        <v>94</v>
+        <v>11</v>
       </c>
       <c r="I29" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="J29" s="12" t="s">
-        <v>76</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="J29" s="12"/>
     </row>
     <row r="30" spans="1:10" ht="60" customHeight="1">
       <c r="A30" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C30" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="B30" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C30" s="6" t="s">
+      <c r="D30" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E30" s="8" t="s">
         <v>101</v>
-      </c>
-      <c r="D30" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E30" s="8" t="s">
-        <v>102</v>
       </c>
       <c r="F30" s="6" t="s">
         <v>11</v>
@@ -2333,30 +2346,30 @@
         <v/>
       </c>
       <c r="H30" s="10" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="I30" s="11" t="s">
-        <v>85</v>
+        <v>25</v>
       </c>
       <c r="J30" s="12" t="s">
-        <v>86</v>
+        <v>26</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="60" customHeight="1">
       <c r="A31" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D31" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E31" s="8" t="s">
         <v>103</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D31" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E31" s="8" t="s">
-        <v>104</v>
       </c>
       <c r="F31" s="6" t="s">
         <v>11</v>
@@ -2366,30 +2379,30 @@
         <v/>
       </c>
       <c r="H31" s="10" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I31" s="11" t="s">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="J31" s="12" t="s">
-        <v>76</v>
+        <v>26</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="60" customHeight="1">
       <c r="A32" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D32" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E32" s="8" t="s">
         <v>105</v>
-      </c>
-      <c r="B32" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C32" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D32" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E32" s="8" t="s">
-        <v>106</v>
       </c>
       <c r="F32" s="6" t="s">
         <v>11</v>
@@ -2399,28 +2412,30 @@
         <v/>
       </c>
       <c r="H32" s="10" t="s">
-        <v>11</v>
+        <v>102</v>
       </c>
       <c r="I32" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="J32" s="12"/>
+        <v>50</v>
+      </c>
+      <c r="J32" s="12" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="33" spans="1:10" ht="60" customHeight="1">
       <c r="A33" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D33" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E33" s="8" t="s">
         <v>107</v>
-      </c>
-      <c r="B33" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C33" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D33" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E33" s="8" t="s">
-        <v>108</v>
       </c>
       <c r="F33" s="6" t="s">
         <v>11</v>
@@ -2430,22 +2445,24 @@
         <v/>
       </c>
       <c r="H33" s="10" t="s">
-        <v>11</v>
+        <v>102</v>
       </c>
       <c r="I33" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="J33" s="12"/>
+        <v>83</v>
+      </c>
+      <c r="J33" s="12" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="34" spans="1:10" ht="60" customHeight="1">
       <c r="A34" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C34" s="6" t="s">
         <v>109</v>
-      </c>
-      <c r="B34" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>68</v>
       </c>
       <c r="D34" s="7" t="s">
         <v>11</v>
@@ -2461,13 +2478,13 @@
         <v/>
       </c>
       <c r="H34" s="10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I34" s="11" t="s">
-        <v>24</v>
+        <v>93</v>
       </c>
       <c r="J34" s="12" t="s">
-        <v>25</v>
+        <v>94</v>
       </c>
     </row>
     <row r="35" spans="1:10" ht="60" customHeight="1">
@@ -2494,18 +2511,18 @@
         <v/>
       </c>
       <c r="H35" s="10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I35" s="11" t="s">
-        <v>114</v>
+        <v>83</v>
       </c>
       <c r="J35" s="12" t="s">
-        <v>115</v>
+        <v>84</v>
       </c>
     </row>
     <row r="36" spans="1:10" ht="60" customHeight="1">
       <c r="A36" s="6" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B36" s="6" t="s">
         <v>11</v>
@@ -2517,7 +2534,7 @@
         <v>11</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="F36" s="6" t="s">
         <v>11</v>
@@ -2527,18 +2544,16 @@
         <v/>
       </c>
       <c r="H36" s="10" t="s">
-        <v>111</v>
+        <v>11</v>
       </c>
       <c r="I36" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="J36" s="12" t="s">
-        <v>86</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="J36" s="12"/>
     </row>
     <row r="37" spans="1:10" ht="60" customHeight="1">
       <c r="A37" s="6" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B37" s="6" t="s">
         <v>11</v>
@@ -2550,7 +2565,7 @@
         <v>11</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="F37" s="6" t="s">
         <v>11</v>
@@ -2560,30 +2575,28 @@
         <v/>
       </c>
       <c r="H37" s="10" t="s">
-        <v>116</v>
+        <v>11</v>
       </c>
       <c r="I37" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="J37" s="12" t="s">
-        <v>76</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="J37" s="12"/>
     </row>
     <row r="38" spans="1:10" ht="60" customHeight="1">
       <c r="A38" s="6" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B38" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>11</v>
+        <v>76</v>
       </c>
       <c r="D38" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="F38" s="6" t="s">
         <v>11</v>
@@ -2593,16 +2606,18 @@
         <v/>
       </c>
       <c r="H38" s="10" t="s">
-        <v>11</v>
+        <v>115</v>
       </c>
       <c r="I38" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="J38" s="12"/>
+        <v>30</v>
+      </c>
+      <c r="J38" s="12" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="39" spans="1:10" ht="60" customHeight="1">
       <c r="A39" s="6" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B39" s="6" t="s">
         <v>11</v>
@@ -2614,7 +2629,7 @@
         <v>11</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="F39" s="6" t="s">
         <v>11</v>
@@ -2624,12 +2639,14 @@
         <v/>
       </c>
       <c r="H39" s="10" t="s">
-        <v>11</v>
+        <v>115</v>
       </c>
       <c r="I39" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="J39" s="12"/>
+        <v>122</v>
+      </c>
+      <c r="J39" s="12" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="40" spans="1:10" ht="60" customHeight="1">
       <c r="A40" s="6" t="s">
@@ -2655,12 +2672,14 @@
         <v/>
       </c>
       <c r="H40" s="10" t="s">
-        <v>11</v>
+        <v>119</v>
       </c>
       <c r="I40" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="J40" s="12"/>
+        <v>93</v>
+      </c>
+      <c r="J40" s="12" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="41" spans="1:10" ht="60" customHeight="1">
       <c r="A41" s="6" t="s">
@@ -2670,7 +2689,7 @@
         <v>11</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="D41" s="7" t="s">
         <v>11</v>
@@ -2689,10 +2708,10 @@
         <v>124</v>
       </c>
       <c r="I41" s="11" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="J41" s="12" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="42" spans="1:10" ht="60" customHeight="1">
@@ -2719,10 +2738,10 @@
         <v/>
       </c>
       <c r="H42" s="10" t="s">
-        <v>130</v>
+        <v>11</v>
       </c>
       <c r="I42" s="11" t="s">
-        <v>131</v>
+        <v>11</v>
       </c>
       <c r="J42" s="12"/>
     </row>
@@ -2734,13 +2753,13 @@
         <v>11</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>60</v>
+        <v>11</v>
       </c>
       <c r="D43" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F43" s="6" t="s">
         <v>11</v>
@@ -2750,30 +2769,28 @@
         <v/>
       </c>
       <c r="H43" s="10" t="s">
-        <v>128</v>
+        <v>11</v>
       </c>
       <c r="I43" s="11" t="s">
-        <v>134</v>
-      </c>
-      <c r="J43" s="12" t="s">
-        <v>135</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="J43" s="12"/>
     </row>
     <row r="44" spans="1:10" ht="60" customHeight="1">
       <c r="A44" s="6" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="B44" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>11</v>
+        <v>47</v>
       </c>
       <c r="D44" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E44" s="8" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="F44" s="6" t="s">
         <v>11</v>
@@ -2783,16 +2800,18 @@
         <v/>
       </c>
       <c r="H44" s="10" t="s">
-        <v>11</v>
+        <v>130</v>
       </c>
       <c r="I44" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="J44" s="12"/>
+        <v>88</v>
+      </c>
+      <c r="J44" s="12" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="45" spans="1:10" ht="60" customHeight="1">
       <c r="A45" s="6" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="B45" s="6" t="s">
         <v>11</v>
@@ -2804,7 +2823,7 @@
         <v>11</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="F45" s="6" t="s">
         <v>11</v>
@@ -2814,28 +2833,28 @@
         <v/>
       </c>
       <c r="H45" s="10" t="s">
-        <v>11</v>
+        <v>136</v>
       </c>
       <c r="I45" s="11" t="s">
-        <v>11</v>
+        <v>137</v>
       </c>
       <c r="J45" s="12"/>
     </row>
     <row r="46" spans="1:10" ht="60" customHeight="1">
       <c r="A46" s="6" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="B46" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>41</v>
+        <v>68</v>
       </c>
       <c r="D46" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E46" s="8" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="F46" s="6" t="s">
         <v>11</v>
@@ -2845,13 +2864,13 @@
         <v/>
       </c>
       <c r="H46" s="10" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="I46" s="11" t="s">
-        <v>80</v>
+        <v>140</v>
       </c>
       <c r="J46" s="12" t="s">
-        <v>81</v>
+        <v>141</v>
       </c>
     </row>
     <row r="47" spans="1:10" ht="60" customHeight="1">
@@ -2878,10 +2897,10 @@
         <v/>
       </c>
       <c r="H47" s="10" t="s">
-        <v>144</v>
+        <v>11</v>
       </c>
       <c r="I47" s="11" t="s">
-        <v>131</v>
+        <v>11</v>
       </c>
       <c r="J47" s="12"/>
     </row>
@@ -2924,7 +2943,7 @@
         <v>11</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>16</v>
+        <v>47</v>
       </c>
       <c r="D49" s="7" t="s">
         <v>11</v>
@@ -2943,10 +2962,10 @@
         <v>144</v>
       </c>
       <c r="I49" s="11" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="J49" s="12" t="s">
-        <v>20</v>
+        <v>89</v>
       </c>
     </row>
     <row r="50" spans="1:10" ht="60" customHeight="1">
@@ -2973,10 +2992,10 @@
         <v/>
       </c>
       <c r="H50" s="10" t="s">
-        <v>11</v>
+        <v>150</v>
       </c>
       <c r="I50" s="11" t="s">
-        <v>11</v>
+        <v>137</v>
       </c>
       <c r="J50" s="12"/>
     </row>
@@ -3019,7 +3038,7 @@
         <v>11</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="D52" s="7" t="s">
         <v>11</v>
@@ -3038,10 +3057,10 @@
         <v>150</v>
       </c>
       <c r="I52" s="11" t="s">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="J52" s="12" t="s">
-        <v>45</v>
+        <v>26</v>
       </c>
     </row>
     <row r="53" spans="1:10" ht="60" customHeight="1">
@@ -3052,13 +3071,13 @@
         <v>11</v>
       </c>
       <c r="C53" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D53" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E53" s="8" t="s">
         <v>155</v>
-      </c>
-      <c r="D53" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E53" s="8" t="s">
-        <v>156</v>
       </c>
       <c r="F53" s="6" t="s">
         <v>11</v>
@@ -3068,18 +3087,16 @@
         <v/>
       </c>
       <c r="H53" s="10" t="s">
-        <v>152</v>
+        <v>11</v>
       </c>
       <c r="I53" s="11" t="s">
-        <v>158</v>
-      </c>
-      <c r="J53" s="12" t="s">
-        <v>159</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="J53" s="12"/>
     </row>
     <row r="54" spans="1:10" ht="60" customHeight="1">
       <c r="A54" s="6" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="B54" s="6" t="s">
         <v>11</v>
@@ -3091,7 +3108,7 @@
         <v>11</v>
       </c>
       <c r="E54" s="8" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="F54" s="6" t="s">
         <v>11</v>
@@ -3101,30 +3118,28 @@
         <v/>
       </c>
       <c r="H54" s="10" t="s">
-        <v>154</v>
+        <v>11</v>
       </c>
       <c r="I54" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="J54" s="12" t="s">
-        <v>76</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="J54" s="12"/>
     </row>
     <row r="55" spans="1:10" ht="60" customHeight="1">
       <c r="A55" s="6" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="B55" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="D55" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E55" s="8" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="F55" s="6" t="s">
         <v>11</v>
@@ -3134,30 +3149,30 @@
         <v/>
       </c>
       <c r="H55" s="10" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="I55" s="11" t="s">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="J55" s="12" t="s">
-        <v>81</v>
+        <v>51</v>
       </c>
     </row>
     <row r="56" spans="1:10" ht="60" customHeight="1">
       <c r="A56" s="6" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="B56" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="D56" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E56" s="8" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="F56" s="6" t="s">
         <v>11</v>
@@ -3167,30 +3182,30 @@
         <v/>
       </c>
       <c r="H56" s="10" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="I56" s="11" t="s">
-        <v>24</v>
+        <v>164</v>
       </c>
       <c r="J56" s="12" t="s">
-        <v>25</v>
+        <v>165</v>
       </c>
     </row>
     <row r="57" spans="1:10" ht="60" customHeight="1">
       <c r="A57" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D57" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E57" s="8" t="s">
         <v>167</v>
-      </c>
-      <c r="B57" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C57" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D57" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E57" s="8" t="s">
-        <v>168</v>
       </c>
       <c r="F57" s="6" t="s">
         <v>11</v>
@@ -3200,28 +3215,30 @@
         <v/>
       </c>
       <c r="H57" s="10" t="s">
-        <v>11</v>
+        <v>160</v>
       </c>
       <c r="I57" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="J57" s="12"/>
+        <v>83</v>
+      </c>
+      <c r="J57" s="12" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="58" spans="1:10" ht="60" customHeight="1">
       <c r="A58" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="B58" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C58" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D58" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E58" s="8" t="s">
         <v>169</v>
-      </c>
-      <c r="B58" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C58" s="6" t="s">
-        <v>170</v>
-      </c>
-      <c r="D58" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E58" s="8" t="s">
-        <v>171</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>11</v>
@@ -3231,30 +3248,30 @@
         <v/>
       </c>
       <c r="H58" s="10" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I58" s="11" t="s">
-        <v>55</v>
+        <v>88</v>
       </c>
       <c r="J58" s="12" t="s">
-        <v>56</v>
+        <v>89</v>
       </c>
     </row>
     <row r="59" spans="1:10" ht="60" customHeight="1">
       <c r="A59" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="D59" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E59" s="8" t="s">
         <v>172</v>
-      </c>
-      <c r="B59" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C59" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="D59" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E59" s="8" t="s">
-        <v>174</v>
       </c>
       <c r="F59" s="6" t="s">
         <v>11</v>
@@ -3264,18 +3281,18 @@
         <v/>
       </c>
       <c r="H59" s="10" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="I59" s="11" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="J59" s="12" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
     </row>
     <row r="60" spans="1:10" ht="60" customHeight="1">
       <c r="A60" s="6" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B60" s="6" t="s">
         <v>11</v>
@@ -3287,7 +3304,7 @@
         <v>11</v>
       </c>
       <c r="E60" s="8" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="F60" s="6" t="s">
         <v>11</v>
@@ -3306,19 +3323,19 @@
     </row>
     <row r="61" spans="1:10" ht="60" customHeight="1">
       <c r="A61" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C61" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="D61" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E61" s="8" t="s">
         <v>177</v>
-      </c>
-      <c r="B61" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C61" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="D61" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E61" s="8" t="s">
-        <v>179</v>
       </c>
       <c r="F61" s="6" t="s">
         <v>11</v>
@@ -3328,30 +3345,30 @@
         <v/>
       </c>
       <c r="H61" s="10" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="I61" s="11" t="s">
-        <v>181</v>
+        <v>63</v>
       </c>
       <c r="J61" s="12" t="s">
-        <v>182</v>
+        <v>64</v>
       </c>
     </row>
     <row r="62" spans="1:10" ht="60" customHeight="1">
       <c r="A62" s="6" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="B62" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>11</v>
+        <v>179</v>
       </c>
       <c r="D62" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E62" s="8" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="F62" s="6" t="s">
         <v>11</v>
@@ -3361,18 +3378,18 @@
         <v/>
       </c>
       <c r="H62" s="10" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="I62" s="11" t="s">
-        <v>80</v>
+        <v>25</v>
       </c>
       <c r="J62" s="12" t="s">
-        <v>81</v>
+        <v>26</v>
       </c>
     </row>
     <row r="63" spans="1:10" ht="60" customHeight="1">
       <c r="A63" s="6" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="B63" s="6" t="s">
         <v>11</v>
@@ -3384,7 +3401,7 @@
         <v>11</v>
       </c>
       <c r="E63" s="8" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="F63" s="6" t="s">
         <v>11</v>
@@ -3403,19 +3420,19 @@
     </row>
     <row r="64" spans="1:10" ht="60" customHeight="1">
       <c r="A64" s="6" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="B64" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>11</v>
+        <v>184</v>
       </c>
       <c r="D64" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E64" s="8" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="F64" s="6" t="s">
         <v>11</v>
@@ -3425,12 +3442,14 @@
         <v/>
       </c>
       <c r="H64" s="10" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="I64" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="J64" s="12"/>
+        <v>187</v>
+      </c>
+      <c r="J64" s="12" t="s">
+        <v>188</v>
+      </c>
     </row>
     <row r="65" spans="1:10" ht="60" customHeight="1">
       <c r="A65" s="6" t="s">
@@ -3456,12 +3475,14 @@
         <v/>
       </c>
       <c r="H65" s="10" t="s">
-        <v>11</v>
+        <v>183</v>
       </c>
       <c r="I65" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="J65" s="12"/>
+        <v>88</v>
+      </c>
+      <c r="J65" s="12" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="66" spans="1:10" ht="60" customHeight="1">
       <c r="A66" s="6" t="s">
@@ -3502,7 +3523,7 @@
         <v>11</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>170</v>
+        <v>11</v>
       </c>
       <c r="D67" s="7" t="s">
         <v>11</v>
@@ -3518,14 +3539,12 @@
         <v/>
       </c>
       <c r="H67" s="10" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="I67" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="J67" s="12" t="s">
-        <v>56</v>
-      </c>
+        <v>137</v>
+      </c>
+      <c r="J67" s="12"/>
     </row>
     <row r="68" spans="1:10" ht="60" customHeight="1">
       <c r="A68" s="6" t="s">
@@ -3535,7 +3554,7 @@
         <v>11</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>68</v>
+        <v>11</v>
       </c>
       <c r="D68" s="7" t="s">
         <v>11</v>
@@ -3551,14 +3570,12 @@
         <v/>
       </c>
       <c r="H68" s="10" t="s">
-        <v>193</v>
+        <v>11</v>
       </c>
       <c r="I68" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="J68" s="12" t="s">
-        <v>25</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="J68" s="12"/>
     </row>
     <row r="69" spans="1:10" ht="60" customHeight="1">
       <c r="A69" s="6" t="s">
@@ -3568,13 +3585,13 @@
         <v>11</v>
       </c>
       <c r="C69" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D69" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E69" s="8" t="s">
         <v>198</v>
-      </c>
-      <c r="D69" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E69" s="8" t="s">
-        <v>199</v>
       </c>
       <c r="F69" s="6" t="s">
         <v>11</v>
@@ -3584,30 +3601,28 @@
         <v/>
       </c>
       <c r="H69" s="10" t="s">
-        <v>195</v>
+        <v>11</v>
       </c>
       <c r="I69" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="J69" s="12" t="s">
-        <v>76</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="J69" s="12"/>
     </row>
     <row r="70" spans="1:10" ht="60" customHeight="1">
       <c r="A70" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="B70" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C70" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="D70" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E70" s="8" t="s">
         <v>200</v>
-      </c>
-      <c r="B70" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C70" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D70" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E70" s="8" t="s">
-        <v>201</v>
       </c>
       <c r="F70" s="6" t="s">
         <v>11</v>
@@ -3617,28 +3632,30 @@
         <v/>
       </c>
       <c r="H70" s="10" t="s">
-        <v>11</v>
+        <v>195</v>
       </c>
       <c r="I70" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="J70" s="12"/>
+        <v>63</v>
+      </c>
+      <c r="J70" s="12" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="71" spans="1:10" ht="60" customHeight="1">
       <c r="A71" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="B71" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C71" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="D71" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E71" s="8" t="s">
         <v>202</v>
-      </c>
-      <c r="B71" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C71" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D71" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E71" s="8" t="s">
-        <v>203</v>
       </c>
       <c r="F71" s="6" t="s">
         <v>11</v>
@@ -3648,22 +3665,24 @@
         <v/>
       </c>
       <c r="H71" s="10" t="s">
-        <v>11</v>
+        <v>199</v>
       </c>
       <c r="I71" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="J71" s="12"/>
+        <v>30</v>
+      </c>
+      <c r="J71" s="12" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="72" spans="1:10" ht="60" customHeight="1">
       <c r="A72" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="B72" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C72" s="6" t="s">
         <v>204</v>
-      </c>
-      <c r="B72" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C72" s="6" t="s">
-        <v>11</v>
       </c>
       <c r="D72" s="7" t="s">
         <v>11</v>
@@ -3679,12 +3698,14 @@
         <v/>
       </c>
       <c r="H72" s="10" t="s">
-        <v>11</v>
+        <v>201</v>
       </c>
       <c r="I72" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="J72" s="12"/>
+        <v>83</v>
+      </c>
+      <c r="J72" s="12" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="73" spans="1:10" ht="60" customHeight="1">
       <c r="A73" s="6" t="s">
@@ -3694,7 +3715,7 @@
         <v>11</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>68</v>
+        <v>11</v>
       </c>
       <c r="D73" s="7" t="s">
         <v>11</v>
@@ -3710,14 +3731,12 @@
         <v/>
       </c>
       <c r="H73" s="10" t="s">
-        <v>202</v>
+        <v>11</v>
       </c>
       <c r="I73" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="J73" s="12" t="s">
-        <v>20</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="J73" s="12"/>
     </row>
     <row r="74" spans="1:10" ht="60" customHeight="1">
       <c r="A74" s="6" t="s">
@@ -3758,7 +3777,7 @@
         <v>11</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="D75" s="7" t="s">
         <v>11</v>
@@ -3774,13 +3793,13 @@
         <v/>
       </c>
       <c r="H75" s="10" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="I75" s="11" t="s">
-        <v>134</v>
+        <v>25</v>
       </c>
       <c r="J75" s="12" t="s">
-        <v>135</v>
+        <v>26</v>
       </c>
     </row>
     <row r="76" spans="1:10" ht="60" customHeight="1">
@@ -3791,7 +3810,7 @@
         <v>11</v>
       </c>
       <c r="C76" s="6" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="D76" s="7" t="s">
         <v>11</v>
@@ -3807,14 +3826,12 @@
         <v/>
       </c>
       <c r="H76" s="10" t="s">
-        <v>210</v>
+        <v>11</v>
       </c>
       <c r="I76" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="J76" s="12" t="s">
-        <v>20</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="J76" s="12"/>
     </row>
     <row r="77" spans="1:10" ht="60" customHeight="1">
       <c r="A77" s="6" t="s">
@@ -3824,7 +3841,7 @@
         <v>11</v>
       </c>
       <c r="C77" s="6" t="s">
-        <v>11</v>
+        <v>68</v>
       </c>
       <c r="D77" s="7" t="s">
         <v>11</v>
@@ -3840,30 +3857,30 @@
         <v/>
       </c>
       <c r="H77" s="10" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="I77" s="11" t="s">
-        <v>75</v>
+        <v>140</v>
       </c>
       <c r="J77" s="12" t="s">
-        <v>217</v>
+        <v>141</v>
       </c>
     </row>
     <row r="78" spans="1:10" ht="60" customHeight="1">
       <c r="A78" s="6" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B78" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C78" s="6" t="s">
-        <v>219</v>
+        <v>37</v>
       </c>
       <c r="D78" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E78" s="8" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="F78" s="6" t="s">
         <v>11</v>
@@ -3876,27 +3893,27 @@
         <v>214</v>
       </c>
       <c r="I78" s="11" t="s">
-        <v>80</v>
+        <v>25</v>
       </c>
       <c r="J78" s="12" t="s">
-        <v>81</v>
+        <v>26</v>
       </c>
     </row>
     <row r="79" spans="1:10" ht="60" customHeight="1">
       <c r="A79" s="6" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="B79" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C79" s="6" t="s">
-        <v>222</v>
+        <v>11</v>
       </c>
       <c r="D79" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E79" s="8" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="F79" s="6" t="s">
         <v>11</v>
@@ -3906,30 +3923,30 @@
         <v/>
       </c>
       <c r="H79" s="10" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="I79" s="11" t="s">
-        <v>225</v>
+        <v>83</v>
       </c>
       <c r="J79" s="12" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
     </row>
     <row r="80" spans="1:10" ht="60" customHeight="1">
       <c r="A80" s="6" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="B80" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C80" s="6" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="D80" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E80" s="8" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="F80" s="6" t="s">
         <v>11</v>
@@ -3939,30 +3956,30 @@
         <v/>
       </c>
       <c r="H80" s="10" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="I80" s="11" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="J80" s="12" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
     </row>
     <row r="81" spans="1:10" ht="60" customHeight="1">
       <c r="A81" s="6" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="B81" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C81" s="6" t="s">
-        <v>11</v>
+        <v>226</v>
       </c>
       <c r="D81" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E81" s="8" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="F81" s="6" t="s">
         <v>11</v>
@@ -3972,12 +3989,14 @@
         <v/>
       </c>
       <c r="H81" s="10" t="s">
-        <v>11</v>
+        <v>222</v>
       </c>
       <c r="I81" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="J81" s="12"/>
+        <v>229</v>
+      </c>
+      <c r="J81" s="12" t="s">
+        <v>230</v>
+      </c>
     </row>
     <row r="82" spans="1:10" ht="60" customHeight="1">
       <c r="A82" s="6" t="s">
@@ -4018,7 +4037,7 @@
         <v>11</v>
       </c>
       <c r="C83" s="6" t="s">
-        <v>31</v>
+        <v>223</v>
       </c>
       <c r="D83" s="7" t="s">
         <v>11</v>
@@ -4034,13 +4053,13 @@
         <v/>
       </c>
       <c r="H83" s="10" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="I83" s="11" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="J83" s="12" t="s">
-        <v>20</v>
+        <v>89</v>
       </c>
     </row>
     <row r="84" spans="1:10" ht="60" customHeight="1">
@@ -4051,7 +4070,7 @@
         <v>11</v>
       </c>
       <c r="C84" s="6" t="s">
-        <v>60</v>
+        <v>11</v>
       </c>
       <c r="D84" s="7" t="s">
         <v>11</v>
@@ -4067,14 +4086,12 @@
         <v/>
       </c>
       <c r="H84" s="10" t="s">
-        <v>233</v>
+        <v>11</v>
       </c>
       <c r="I84" s="11" t="s">
-        <v>134</v>
-      </c>
-      <c r="J84" s="12" t="s">
-        <v>135</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="J84" s="12"/>
     </row>
     <row r="85" spans="1:10" ht="60" customHeight="1">
       <c r="A85" s="6" t="s">
@@ -4084,7 +4101,7 @@
         <v>11</v>
       </c>
       <c r="C85" s="6" t="s">
-        <v>178</v>
+        <v>11</v>
       </c>
       <c r="D85" s="7" t="s">
         <v>11</v>
@@ -4100,14 +4117,12 @@
         <v/>
       </c>
       <c r="H85" s="10" t="s">
-        <v>235</v>
+        <v>11</v>
       </c>
       <c r="I85" s="11" t="s">
-        <v>225</v>
-      </c>
-      <c r="J85" s="12" t="s">
-        <v>226</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="J85" s="12"/>
     </row>
     <row r="86" spans="1:10" ht="60" customHeight="1">
       <c r="A86" s="6" t="s">
@@ -4117,7 +4132,7 @@
         <v>11</v>
       </c>
       <c r="C86" s="6" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="D86" s="7" t="s">
         <v>11</v>
@@ -4136,10 +4151,10 @@
         <v>237</v>
       </c>
       <c r="I86" s="11" t="s">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="J86" s="12" t="s">
-        <v>217</v>
+        <v>26</v>
       </c>
     </row>
     <row r="87" spans="1:10" ht="60" customHeight="1">
@@ -4150,7 +4165,7 @@
         <v>11</v>
       </c>
       <c r="C87" s="6" t="s">
-        <v>11</v>
+        <v>68</v>
       </c>
       <c r="D87" s="7" t="s">
         <v>11</v>
@@ -4166,13 +4181,13 @@
         <v/>
       </c>
       <c r="H87" s="10" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="I87" s="11" t="s">
-        <v>80</v>
+        <v>140</v>
       </c>
       <c r="J87" s="12" t="s">
-        <v>81</v>
+        <v>141</v>
       </c>
     </row>
     <row r="88" spans="1:10" ht="60" customHeight="1">
@@ -4183,7 +4198,7 @@
         <v>11</v>
       </c>
       <c r="C88" s="6" t="s">
-        <v>198</v>
+        <v>184</v>
       </c>
       <c r="D88" s="7" t="s">
         <v>11</v>
@@ -4202,10 +4217,10 @@
         <v>241</v>
       </c>
       <c r="I88" s="11" t="s">
-        <v>75</v>
+        <v>229</v>
       </c>
       <c r="J88" s="12" t="s">
-        <v>76</v>
+        <v>230</v>
       </c>
     </row>
     <row r="89" spans="1:10" ht="60" customHeight="1">
@@ -4232,12 +4247,14 @@
         <v/>
       </c>
       <c r="H89" s="10" t="s">
-        <v>11</v>
+        <v>243</v>
       </c>
       <c r="I89" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="J89" s="12"/>
+        <v>83</v>
+      </c>
+      <c r="J89" s="12" t="s">
+        <v>221</v>
+      </c>
     </row>
     <row r="90" spans="1:10" ht="60" customHeight="1">
       <c r="A90" s="6" t="s">
@@ -4263,12 +4280,14 @@
         <v/>
       </c>
       <c r="H90" s="10" t="s">
-        <v>11</v>
+        <v>241</v>
       </c>
       <c r="I90" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="J90" s="12"/>
+        <v>88</v>
+      </c>
+      <c r="J90" s="12" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="91" spans="1:10" ht="60" customHeight="1">
       <c r="A91" s="6" t="s">
@@ -4278,7 +4297,7 @@
         <v>11</v>
       </c>
       <c r="C91" s="6" t="s">
-        <v>11</v>
+        <v>204</v>
       </c>
       <c r="D91" s="7" t="s">
         <v>11</v>
@@ -4297,10 +4316,10 @@
         <v>247</v>
       </c>
       <c r="I91" s="11" t="s">
-        <v>225</v>
+        <v>83</v>
       </c>
       <c r="J91" s="12" t="s">
-        <v>226</v>
+        <v>84</v>
       </c>
     </row>
     <row r="92" spans="1:10" ht="60" customHeight="1">
@@ -4311,7 +4330,7 @@
         <v>11</v>
       </c>
       <c r="C92" s="6" t="s">
-        <v>170</v>
+        <v>11</v>
       </c>
       <c r="D92" s="7" t="s">
         <v>11</v>
@@ -4327,14 +4346,12 @@
         <v/>
       </c>
       <c r="H92" s="10" t="s">
-        <v>249</v>
+        <v>11</v>
       </c>
       <c r="I92" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="J92" s="12" t="s">
-        <v>56</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="J92" s="12"/>
     </row>
     <row r="93" spans="1:10" ht="60" customHeight="1">
       <c r="A93" s="6" t="s">
@@ -4344,13 +4361,13 @@
         <v>11</v>
       </c>
       <c r="C93" s="6" t="s">
-        <v>68</v>
+        <v>11</v>
       </c>
       <c r="D93" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E93" s="8" t="s">
-        <v>254</v>
+        <v>56</v>
       </c>
       <c r="F93" s="6" t="s">
         <v>11</v>
@@ -4360,30 +4377,28 @@
         <v/>
       </c>
       <c r="H93" s="10" t="s">
-        <v>251</v>
+        <v>11</v>
       </c>
       <c r="I93" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="J93" s="12" t="s">
-        <v>25</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="J93" s="12"/>
     </row>
     <row r="94" spans="1:10" ht="60" customHeight="1">
       <c r="A94" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="B94" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C94" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D94" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E94" s="8" t="s">
         <v>255</v>
-      </c>
-      <c r="B94" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C94" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="D94" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E94" s="8" t="s">
-        <v>256</v>
       </c>
       <c r="F94" s="6" t="s">
         <v>11</v>
@@ -4393,30 +4408,28 @@
         <v/>
       </c>
       <c r="H94" s="10" t="s">
-        <v>251</v>
+        <v>11</v>
       </c>
       <c r="I94" s="11" t="s">
-        <v>114</v>
-      </c>
-      <c r="J94" s="12" t="s">
-        <v>115</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="J94" s="12"/>
     </row>
     <row r="95" spans="1:10" ht="60" customHeight="1">
       <c r="A95" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="B95" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C95" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D95" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E95" s="8" t="s">
         <v>257</v>
-      </c>
-      <c r="B95" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C95" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="D95" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E95" s="8" t="s">
-        <v>259</v>
       </c>
       <c r="F95" s="6" t="s">
         <v>11</v>
@@ -4426,30 +4439,30 @@
         <v/>
       </c>
       <c r="H95" s="10" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="I95" s="11" t="s">
-        <v>261</v>
+        <v>229</v>
       </c>
       <c r="J95" s="12" t="s">
-        <v>262</v>
+        <v>230</v>
       </c>
     </row>
     <row r="96" spans="1:10" ht="60" customHeight="1">
       <c r="A96" s="6" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="B96" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C96" s="6" t="s">
-        <v>47</v>
+        <v>176</v>
       </c>
       <c r="D96" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E96" s="8" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="F96" s="6" t="s">
         <v>11</v>
@@ -4459,30 +4472,30 @@
         <v/>
       </c>
       <c r="H96" s="10" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="I96" s="11" t="s">
-        <v>85</v>
+        <v>63</v>
       </c>
       <c r="J96" s="12" t="s">
-        <v>86</v>
+        <v>64</v>
       </c>
     </row>
     <row r="97" spans="1:10" ht="60" customHeight="1">
       <c r="A97" s="6" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="B97" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C97" s="6" t="s">
-        <v>47</v>
+        <v>76</v>
       </c>
       <c r="D97" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E97" s="8" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="F97" s="6" t="s">
         <v>11</v>
@@ -4492,30 +4505,30 @@
         <v/>
       </c>
       <c r="H97" s="10" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="I97" s="11" t="s">
-        <v>85</v>
+        <v>30</v>
       </c>
       <c r="J97" s="12" t="s">
-        <v>86</v>
+        <v>31</v>
       </c>
     </row>
     <row r="98" spans="1:10" ht="60" customHeight="1">
       <c r="A98" s="6" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="B98" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C98" s="6" t="s">
-        <v>11</v>
+        <v>109</v>
       </c>
       <c r="D98" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E98" s="8" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="F98" s="6" t="s">
         <v>11</v>
@@ -4525,28 +4538,30 @@
         <v/>
       </c>
       <c r="H98" s="10" t="s">
-        <v>11</v>
+        <v>258</v>
       </c>
       <c r="I98" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="J98" s="12"/>
+        <v>122</v>
+      </c>
+      <c r="J98" s="12" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="99" spans="1:10" ht="60" customHeight="1">
       <c r="A99" s="6" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="B99" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C99" s="6" t="s">
-        <v>41</v>
+        <v>265</v>
       </c>
       <c r="D99" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E99" s="8" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="F99" s="6" t="s">
         <v>11</v>
@@ -4556,30 +4571,30 @@
         <v/>
       </c>
       <c r="H99" s="10" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="I99" s="11" t="s">
-        <v>80</v>
+        <v>268</v>
       </c>
       <c r="J99" s="12" t="s">
-        <v>81</v>
+        <v>269</v>
       </c>
     </row>
     <row r="100" spans="1:10" ht="60" customHeight="1">
       <c r="A100" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="B100" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C100" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D100" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E100" s="8" t="s">
         <v>271</v>
-      </c>
-      <c r="B100" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C100" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="D100" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E100" s="8" t="s">
-        <v>272</v>
       </c>
       <c r="F100" s="6" t="s">
         <v>11</v>
@@ -4589,30 +4604,30 @@
         <v/>
       </c>
       <c r="H100" s="10" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="I100" s="11" t="s">
-        <v>24</v>
+        <v>93</v>
       </c>
       <c r="J100" s="12" t="s">
-        <v>25</v>
+        <v>94</v>
       </c>
     </row>
     <row r="101" spans="1:10" ht="60" customHeight="1">
       <c r="A101" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="B101" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C101" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D101" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E101" s="8" t="s">
         <v>273</v>
-      </c>
-      <c r="B101" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C101" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="D101" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E101" s="8" t="s">
-        <v>274</v>
       </c>
       <c r="F101" s="6" t="s">
         <v>11</v>
@@ -4622,30 +4637,28 @@
         <v/>
       </c>
       <c r="H101" s="10" t="s">
-        <v>271</v>
+        <v>11</v>
       </c>
       <c r="I101" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="J101" s="12" t="s">
-        <v>25</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="J101" s="12"/>
     </row>
     <row r="102" spans="1:10" ht="60" customHeight="1">
       <c r="A102" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="B102" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C102" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D102" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E102" s="8" t="s">
         <v>275</v>
-      </c>
-      <c r="B102" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C102" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D102" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E102" s="8" t="s">
-        <v>276</v>
       </c>
       <c r="F102" s="6" t="s">
         <v>11</v>
@@ -4655,28 +4668,30 @@
         <v/>
       </c>
       <c r="H102" s="10" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="I102" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="J102" s="12"/>
+        <v>88</v>
+      </c>
+      <c r="J102" s="12" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="103" spans="1:10" ht="60" customHeight="1">
       <c r="A103" s="6" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="B103" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C103" s="6" t="s">
-        <v>11</v>
+        <v>76</v>
       </c>
       <c r="D103" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E103" s="8" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="F103" s="6" t="s">
         <v>11</v>
@@ -4686,28 +4701,30 @@
         <v/>
       </c>
       <c r="H103" s="10" t="s">
-        <v>11</v>
+        <v>274</v>
       </c>
       <c r="I103" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="J103" s="12"/>
+        <v>30</v>
+      </c>
+      <c r="J103" s="12" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="104" spans="1:10" ht="60" customHeight="1">
       <c r="A104" s="6" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B104" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C104" s="6" t="s">
-        <v>11</v>
+        <v>76</v>
       </c>
       <c r="D104" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E104" s="8" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F104" s="6" t="s">
         <v>11</v>
@@ -4717,28 +4734,30 @@
         <v/>
       </c>
       <c r="H104" s="10" t="s">
-        <v>11</v>
+        <v>276</v>
       </c>
       <c r="I104" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="J104" s="12"/>
+        <v>30</v>
+      </c>
+      <c r="J104" s="12" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="105" spans="1:10" ht="60" customHeight="1">
       <c r="A105" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="B105" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C105" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D105" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E105" s="8" t="s">
         <v>281</v>
-      </c>
-      <c r="B105" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C105" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D105" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E105" s="8" t="s">
-        <v>282</v>
       </c>
       <c r="F105" s="6" t="s">
         <v>11</v>
@@ -4748,28 +4767,28 @@
         <v/>
       </c>
       <c r="H105" s="10" t="s">
-        <v>11</v>
+        <v>282</v>
       </c>
       <c r="I105" s="11" t="s">
-        <v>11</v>
+        <v>137</v>
       </c>
       <c r="J105" s="12"/>
     </row>
     <row r="106" spans="1:10" ht="60" customHeight="1">
       <c r="A106" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="B106" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C106" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D106" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E106" s="8" t="s">
         <v>283</v>
-      </c>
-      <c r="B106" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C106" s="6" t="s">
-        <v>284</v>
-      </c>
-      <c r="D106" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E106" s="8" t="s">
-        <v>285</v>
       </c>
       <c r="F106" s="6" t="s">
         <v>11</v>
@@ -4779,18 +4798,16 @@
         <v/>
       </c>
       <c r="H106" s="10" t="s">
-        <v>281</v>
+        <v>11</v>
       </c>
       <c r="I106" s="11" t="s">
-        <v>287</v>
-      </c>
-      <c r="J106" s="12" t="s">
-        <v>288</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="J106" s="12"/>
     </row>
     <row r="107" spans="1:10" ht="60" customHeight="1">
       <c r="A107" s="6" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="B107" s="6" t="s">
         <v>11</v>
@@ -4802,7 +4819,7 @@
         <v>11</v>
       </c>
       <c r="E107" s="8" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="F107" s="6" t="s">
         <v>11</v>
@@ -4821,19 +4838,19 @@
     </row>
     <row r="108" spans="1:10" ht="60" customHeight="1">
       <c r="A108" s="6" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="B108" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C108" s="6" t="s">
-        <v>11</v>
+        <v>287</v>
       </c>
       <c r="D108" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E108" s="8" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="F108" s="6" t="s">
         <v>11</v>
@@ -4843,28 +4860,30 @@
         <v/>
       </c>
       <c r="H108" s="10" t="s">
-        <v>11</v>
+        <v>284</v>
       </c>
       <c r="I108" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="J108" s="12"/>
+        <v>290</v>
+      </c>
+      <c r="J108" s="12" t="s">
+        <v>291</v>
+      </c>
     </row>
     <row r="109" spans="1:10" ht="60" customHeight="1">
       <c r="A109" s="6" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B109" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C109" s="6" t="s">
-        <v>294</v>
+        <v>11</v>
       </c>
       <c r="D109" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E109" s="8" t="s">
-        <v>295</v>
+        <v>56</v>
       </c>
       <c r="F109" s="6" t="s">
         <v>11</v>
@@ -4874,18 +4893,16 @@
         <v/>
       </c>
       <c r="H109" s="10" t="s">
-        <v>291</v>
+        <v>11</v>
       </c>
       <c r="I109" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="J109" s="12" t="s">
-        <v>20</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="J109" s="12"/>
     </row>
     <row r="110" spans="1:10" ht="60" customHeight="1">
       <c r="A110" s="6" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="B110" s="6" t="s">
         <v>11</v>
@@ -4897,7 +4914,7 @@
         <v>11</v>
       </c>
       <c r="E110" s="8" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="F110" s="6" t="s">
         <v>11</v>
@@ -4916,7 +4933,7 @@
     </row>
     <row r="111" spans="1:10" ht="60" customHeight="1">
       <c r="A111" s="6" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="B111" s="6" t="s">
         <v>11</v>
@@ -4928,7 +4945,7 @@
         <v>11</v>
       </c>
       <c r="E111" s="8" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="F111" s="6" t="s">
         <v>11</v>
@@ -4947,19 +4964,19 @@
     </row>
     <row r="112" spans="1:10" ht="60" customHeight="1">
       <c r="A112" s="6" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="B112" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C112" s="6" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="D112" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E112" s="8" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="F112" s="6" t="s">
         <v>11</v>
@@ -4969,30 +4986,30 @@
         <v/>
       </c>
       <c r="H112" s="10" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="I112" s="11" t="s">
-        <v>261</v>
+        <v>25</v>
       </c>
       <c r="J112" s="12" t="s">
-        <v>262</v>
+        <v>26</v>
       </c>
     </row>
     <row r="113" spans="1:10" ht="60" customHeight="1">
       <c r="A113" s="6" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="B113" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C113" s="6" t="s">
-        <v>68</v>
+        <v>11</v>
       </c>
       <c r="D113" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E113" s="8" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="F113" s="6" t="s">
         <v>11</v>
@@ -5002,30 +5019,28 @@
         <v/>
       </c>
       <c r="H113" s="10" t="s">
-        <v>300</v>
+        <v>11</v>
       </c>
       <c r="I113" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="J113" s="12" t="s">
-        <v>25</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="J113" s="12"/>
     </row>
     <row r="114" spans="1:10" ht="60" customHeight="1">
       <c r="A114" s="6" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="B114" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C114" s="6" t="s">
-        <v>68</v>
+        <v>11</v>
       </c>
       <c r="D114" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E114" s="8" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="F114" s="6" t="s">
         <v>11</v>
@@ -5035,18 +5050,16 @@
         <v/>
       </c>
       <c r="H114" s="10" t="s">
-        <v>303</v>
+        <v>11</v>
       </c>
       <c r="I114" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="J114" s="12" t="s">
-        <v>25</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="J114" s="12"/>
     </row>
     <row r="115" spans="1:10" ht="60" customHeight="1">
       <c r="A115" s="6" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="B115" s="6" t="s">
         <v>11</v>
@@ -5058,7 +5071,7 @@
         <v>11</v>
       </c>
       <c r="E115" s="8" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="F115" s="6" t="s">
         <v>11</v>
@@ -5068,30 +5081,28 @@
         <v/>
       </c>
       <c r="H115" s="10" t="s">
-        <v>303</v>
+        <v>11</v>
       </c>
       <c r="I115" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="J115" s="12" t="s">
-        <v>25</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="J115" s="12"/>
     </row>
     <row r="116" spans="1:10" ht="60" customHeight="1">
       <c r="A116" s="6" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="B116" s="6" t="s">
         <v>11</v>
       </c>
       <c r="C116" s="6" t="s">
-        <v>11</v>
+        <v>307</v>
       </c>
       <c r="D116" s="7" t="s">
         <v>11</v>
       </c>
       <c r="E116" s="8" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="F116" s="6" t="s">
         <v>11</v>
@@ -5101,12 +5112,175 @@
         <v/>
       </c>
       <c r="H116" s="10" t="s">
-        <v>11</v>
+        <v>304</v>
       </c>
       <c r="I116" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="J116" s="12"/>
+        <v>268</v>
+      </c>
+      <c r="J116" s="12" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="117" spans="1:10" ht="60" customHeight="1">
+      <c r="A117" s="6" t="s">
+        <v>309</v>
+      </c>
+      <c r="B117" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C117" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D117" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E117" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="F117" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G117" s="9">
+        <f>IF(A117=1,"_",IF(C117="_","???",C117))</f>
+        <v/>
+      </c>
+      <c r="H117" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="I117" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="J117" s="12"/>
+    </row>
+    <row r="118" spans="1:10" ht="60" customHeight="1">
+      <c r="A118" s="6" t="s">
+        <v>310</v>
+      </c>
+      <c r="B118" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C118" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="D118" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E118" s="8" t="s">
+        <v>311</v>
+      </c>
+      <c r="F118" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G118" s="9">
+        <f>IF(A118=1,"_",IF(C118="_","???",C118))</f>
+        <v/>
+      </c>
+      <c r="H118" s="10" t="s">
+        <v>306</v>
+      </c>
+      <c r="I118" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="J118" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="119" spans="1:10" ht="60" customHeight="1">
+      <c r="A119" s="6" t="s">
+        <v>312</v>
+      </c>
+      <c r="B119" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C119" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="D119" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E119" s="8" t="s">
+        <v>313</v>
+      </c>
+      <c r="F119" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G119" s="9">
+        <f>IF(A119=1,"_",IF(C119="_","???",C119))</f>
+        <v/>
+      </c>
+      <c r="H119" s="10" t="s">
+        <v>310</v>
+      </c>
+      <c r="I119" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="J119" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="120" spans="1:10" ht="60" customHeight="1">
+      <c r="A120" s="6" t="s">
+        <v>314</v>
+      </c>
+      <c r="B120" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C120" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D120" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E120" s="8" t="s">
+        <v>315</v>
+      </c>
+      <c r="F120" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G120" s="9">
+        <f>IF(A120=1,"_",IF(C120="_","???",C120))</f>
+        <v/>
+      </c>
+      <c r="H120" s="10" t="s">
+        <v>310</v>
+      </c>
+      <c r="I120" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="J120" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="121" spans="1:10" ht="60" customHeight="1">
+      <c r="A121" s="6" t="s">
+        <v>316</v>
+      </c>
+      <c r="B121" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C121" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D121" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E121" s="8" t="s">
+        <v>317</v>
+      </c>
+      <c r="F121" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G121" s="9">
+        <f>IF(A121=1,"_",IF(C121="_","???",C121))</f>
+        <v/>
+      </c>
+      <c r="H121" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="I121" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="J121" s="12"/>
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>

</xml_diff>